<commit_message>
effect: unify tag requirement naming and schema
</commit_message>
<xml_diff>
--- a/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.gameplayEffect.xlsx
+++ b/EX_GAS_Config/ProjectConfigTable/exgas_config/Datas/#exgas.gameplayEffect.xlsx
@@ -1379,41 +1379,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr/>
-  <dimension ref="A1:AK26"/>
+  <dimension ref="A1:AG26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="3" max="4" width="12.2166666666667" customWidth="1"/>
     <col min="5" max="5" width="15.6666666666667" customWidth="1"/>
     <col min="6" max="6" width="16.775" customWidth="1"/>
-    <col min="7" max="7" width="28.25" customWidth="1"/>
-    <col min="8" max="9" width="25.775" customWidth="1"/>
-    <col min="10" max="10" width="24.8833333333333" customWidth="1"/>
-    <col min="11" max="11" width="46.25" customWidth="1"/>
-    <col min="12" max="12" width="37" customWidth="1"/>
-    <col min="13" max="13" width="26.5833333333333" customWidth="1"/>
-    <col min="14" max="14" width="18.8833333333333" customWidth="1"/>
-    <col min="15" max="16" width="12.2166666666667" customWidth="1"/>
-    <col min="17" max="17" width="21" customWidth="1"/>
-    <col min="18" max="20" width="14.2166666666667" customWidth="1"/>
+    <col min="7" max="7" width="25.775" customWidth="1"/>
+    <col min="8" max="8" width="24.8833333333333" customWidth="1"/>
+    <col min="9" max="9" width="37" customWidth="1"/>
+    <col min="10" max="10" width="18.8833333333333" customWidth="1"/>
+    <col min="11" max="12" width="12.2166666666667" customWidth="1"/>
+    <col min="13" max="13" width="21" customWidth="1"/>
+    <col min="14" max="16" width="14.2166666666667" customWidth="1"/>
+    <col min="17" max="17" width="15.2166666666667" customWidth="1"/>
+    <col min="18" max="18" width="15" customWidth="1"/>
+    <col min="19" max="19" width="15.1083333333333" customWidth="1"/>
+    <col min="20" max="20" width="13.4416666666667" customWidth="1"/>
     <col min="21" max="21" width="15.2166666666667" customWidth="1"/>
-    <col min="22" max="22" width="15" customWidth="1"/>
-    <col min="23" max="23" width="15.1083333333333" customWidth="1"/>
-    <col min="24" max="24" width="13.4416666666667" customWidth="1"/>
-    <col min="25" max="25" width="15.2166666666667" customWidth="1"/>
-    <col min="26" max="26" width="17.775" customWidth="1"/>
-    <col min="27" max="27" width="18.6666666666667" customWidth="1"/>
-    <col min="28" max="28" width="24.4416666666667" customWidth="1"/>
-    <col min="29" max="29" width="12.2166666666667" customWidth="1"/>
-    <col min="30" max="30" width="11" customWidth="1"/>
-    <col min="31" max="31" width="14.775" customWidth="1"/>
-    <col min="32" max="32" width="19.4416666666667" customWidth="1"/>
-    <col min="33" max="33" width="15.4416666666667" customWidth="1"/>
-    <col min="34" max="34" width="12.2166666666667" customWidth="1"/>
-    <col min="35" max="35" width="17.3333333333333" customWidth="1"/>
-    <col min="36" max="36" width="14.3333333333333" customWidth="1"/>
-    <col min="37" max="37" width="13.1083333333333" customWidth="1"/>
+    <col min="22" max="22" width="17.775" customWidth="1"/>
+    <col min="23" max="23" width="18.6666666666667" customWidth="1"/>
+    <col min="24" max="24" width="24.4416666666667" customWidth="1"/>
+    <col min="25" max="25" width="12.2166666666667" customWidth="1"/>
+    <col min="26" max="26" width="11" customWidth="1"/>
+    <col min="27" max="27" width="14.775" customWidth="1"/>
+    <col min="28" max="28" width="19.4416666666667" customWidth="1"/>
+    <col min="29" max="29" width="15.4416666666667" customWidth="1"/>
+    <col min="30" max="30" width="12.2166666666667" customWidth="1"/>
+    <col min="31" max="31" width="17.3333333333333" customWidth="1"/>
+    <col min="32" max="32" width="14.3333333333333" customWidth="1"/>
+    <col min="33" max="33" width="13.1083333333333" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.2" customHeight="1" spans="1:37">
@@ -1436,60 +1433,48 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="I1" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="U1" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1512,38 +1497,26 @@
       <c r="F2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="K2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="J2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="V2" s="1" t="s">
         <v>28</v>
@@ -1552,22 +1525,30 @@
         <v>28</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AB2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AC2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
         <v>34</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TagRequirementData?</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TagRequirementData?</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>TagRequirementData?</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>TagRequirementData?</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:37">
@@ -1587,98 +1568,94 @@
         <v>39</v>
       </c>
       <c r="F3" s="1"/>
-      <c r="G3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="K3" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="AB3" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="AC3" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="AD3" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="AG3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI3" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AJ3" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="AK3" s="1" t="s">
         <v>70</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>应用GE需要匹配的Tag规则</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>激活GE需要匹配的Tag规则</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>移除匹配Tag规则的Effect</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>免疫GE需要匹配的Tag规则</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:37">
@@ -1698,43 +1675,35 @@
       <c r="F4" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="6" t="s">
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>-1</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>5</v>
+      </c>
+      <c r="O4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P4" t="s">
+        <v>76</v>
+      </c>
+      <c r="R4" t="s">
         <v>73</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="S4" t="s">
         <v>73</v>
       </c>
-      <c r="J4" t="s">
+      <c r="T4" t="s">
         <v>73</v>
       </c>
-      <c r="K4"/>
-      <c r="L4" t="s">
+      <c r="U4" t="s">
         <v>73</v>
-      </c>
-      <c r="M4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" t="s">
-        <v>73</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>-1</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4">
-        <v>5</v>
-      </c>
-      <c r="S4" t="s">
-        <v>75</v>
-      </c>
-      <c r="T4" t="s">
-        <v>76</v>
       </c>
       <c r="V4" t="s">
         <v>73</v>
@@ -1742,20 +1711,8 @@
       <c r="W4" t="s">
         <v>73</v>
       </c>
-      <c r="X4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AB4" s="1"/>
-      <c r="AC4" s="1"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="1"/>
     </row>
     <row r="5" spans="1:37">
       <c r="A5" s="1"/>
@@ -1774,16 +1731,16 @@
       <c r="F5" t="s">
         <v>80</v>
       </c>
-      <c r="O5">
+      <c r="K5">
         <v>0</v>
       </c>
-      <c r="P5">
+      <c r="L5">
         <v>-1</v>
       </c>
-      <c r="Q5" t="b">
+      <c r="M5" t="b">
         <v>0</v>
       </c>
-      <c r="U5" t="s">
+      <c r="Q5" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1800,20 +1757,26 @@
       <c r="E6" t="s">
         <v>79</v>
       </c>
-      <c r="H6" t="s">
-        <v>84</v>
-      </c>
-      <c r="L6" t="s">
-        <v>79</v>
-      </c>
-      <c r="N6" t="s">
-        <v>85</v>
-      </c>
-      <c r="U6" t="s">
+      <c r="Q6" t="s">
         <v>86</v>
       </c>
-      <c r="V6" t="s">
+      <c r="R6" t="s">
         <v>87</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>400;0;0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0;3001;0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0;2004;0</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -1829,44 +1792,53 @@
       <c r="F7" t="s">
         <v>90</v>
       </c>
-      <c r="J7" t="s">
-        <v>91</v>
-      </c>
-      <c r="O7">
+      <c r="K7">
         <v>0</v>
       </c>
-      <c r="P7">
+      <c r="L7">
         <v>600</v>
       </c>
-      <c r="Q7" t="b">
+      <c r="M7" t="b">
         <v>0</v>
       </c>
-      <c r="R7">
+      <c r="N7">
         <v>60</v>
+      </c>
+      <c r="O7" t="s">
+        <v>87</v>
+      </c>
+      <c r="P7" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>92</v>
       </c>
       <c r="S7" t="s">
         <v>87</v>
       </c>
       <c r="T7" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="U7" t="s">
-        <v>92</v>
+        <v>87</v>
+      </c>
+      <c r="V7" t="s">
+        <v>87</v>
       </c>
       <c r="W7" t="s">
         <v>87</v>
       </c>
-      <c r="X7" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z7" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>87</v>
+      <c r="Y7">
+        <v>1</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>10</v>
+      </c>
+      <c r="AB7">
+        <v>1</v>
       </c>
       <c r="AC7">
         <v>1</v>
@@ -1874,26 +1846,19 @@
       <c r="AD7">
         <v>0</v>
       </c>
-      <c r="AE7">
-        <v>10</v>
-      </c>
-      <c r="AF7">
-        <v>1</v>
-      </c>
-      <c r="AG7">
-        <v>1</v>
-      </c>
-      <c r="AH7">
-        <v>0</v>
-      </c>
-      <c r="AI7" t="s">
+      <c r="AE7" t="s">
         <v>93</v>
       </c>
-      <c r="AJ7" t="s">
+      <c r="AF7" t="s">
         <v>93</v>
       </c>
-      <c r="AK7" t="s">
+      <c r="AG7" t="s">
         <v>87</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>200;0;0</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -1906,7 +1871,7 @@
       <c r="D8" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="U8" t="s">
+      <c r="Q8" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1921,22 +1886,22 @@
       <c r="D9" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="O9">
+      <c r="K9">
         <v>0</v>
       </c>
-      <c r="P9">
+      <c r="L9">
         <v>-1</v>
       </c>
-      <c r="Q9" t="b">
+      <c r="M9" t="b">
         <v>0</v>
       </c>
-      <c r="R9">
+      <c r="N9">
         <v>60</v>
       </c>
-      <c r="S9" t="s">
+      <c r="O9" t="s">
         <v>98</v>
       </c>
-      <c r="T9" t="s">
+      <c r="P9" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1950,7 +1915,7 @@
       <c r="D10" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="U10" t="s">
+      <c r="Q10" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1964,10 +1929,10 @@
       <c r="D11" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="U11" t="s">
+      <c r="Q11" t="s">
         <v>102</v>
       </c>
-      <c r="V11" t="s">
+      <c r="R11" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1987,43 +1952,31 @@
       <c r="F12" t="s">
         <v>105</v>
       </c>
-      <c r="H12" t="s">
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>60</v>
+      </c>
+      <c r="M12" t="b">
+        <v>0</v>
+      </c>
+      <c r="R12" t="s">
         <v>73</v>
       </c>
-      <c r="J12" t="s">
+      <c r="S12" t="s">
+        <v>106</v>
+      </c>
+      <c r="T12" t="s">
         <v>73</v>
       </c>
-      <c r="L12" t="s">
+      <c r="U12" t="s">
         <v>73</v>
-      </c>
-      <c r="N12" t="s">
-        <v>73</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
-        <v>60</v>
-      </c>
-      <c r="Q12" t="b">
-        <v>0</v>
       </c>
       <c r="V12" t="s">
         <v>73</v>
       </c>
       <c r="W12" t="s">
-        <v>106</v>
-      </c>
-      <c r="X12" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y12" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>73</v>
-      </c>
-      <c r="AA12" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2037,7 +1990,7 @@
       <c r="D13" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="U13" t="s">
+      <c r="Q13" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2054,13 +2007,13 @@
       <c r="F14" t="s">
         <v>110</v>
       </c>
-      <c r="O14">
+      <c r="K14">
         <v>0</v>
       </c>
-      <c r="P14">
+      <c r="L14">
         <v>-1</v>
       </c>
-      <c r="Q14" t="b">
+      <c r="M14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2074,7 +2027,7 @@
       <c r="D15" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="U15" t="s">
+      <c r="Q15" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2132,6 +2085,6 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing ns1:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>